<commit_message>
Actualizacion por incorporacion de Trafos al pipeline
</commit_message>
<xml_diff>
--- a/data/network_500kv/buses_PSSE_vs_geosadi.xlsx
+++ b/data/network_500kv/buses_PSSE_vs_geosadi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\pypsa-ar-base\data\network_500kv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F89EF16C-B570-4414-8730-F1464458751A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60DBB491-16F3-4429-957F-0151B034CD9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B6A7DE32-F623-4F3B-A33D-1C155ACFA8CC}"/>
   </bookViews>
@@ -2760,10 +2760,10 @@
         <v>67</v>
       </c>
       <c r="D48">
-        <v>-34.752712000000002</v>
+        <v>-34.9118465411849</v>
       </c>
       <c r="E48">
-        <v>-58.542000000000002</v>
+        <v>-58.724642214966202</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>170</v>

</xml_diff>